<commit_message>
Stage 8 fixes: F-014
</commit_message>
<xml_diff>
--- a/output/archive/Archive/Users/langforde_old_laptop/Commercial/2022/early-CMC_rates_060122_EL.xlsx
+++ b/output/archive/Archive/Users/langforde_old_laptop/Commercial/2022/early-CMC_rates_060122_EL.xlsx
@@ -145,7 +145,7 @@
   <commentList>
     <comment ref="C6" authorId="0" shapeId="0">
       <text>
-        <t>Still need the 2021 card figure. Didn't get it from the old folder, will ask Dimitra</t>
+        <t>Still need the 2021 card figure for the excipient line. Didn't get it from the old folder, will ask Dimitra</t>
       </text>
     </comment>
     <comment ref="A10" authorId="0" shapeId="0">
@@ -534,22 +534,20 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Vehicle ladder, work package</t>
+          <t>Vehicle ladder</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>per work package</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
+          <t>per vehicle ladder</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>9850</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Two-week screen, bench sheet per vehicle</t>
+          <t>Two-week screen, bench sheet per vehicle. No volume discount</t>
         </is>
       </c>
     </row>
@@ -787,7 +785,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Julia and Miguel agreed the ladder should be quoted per work package, not per vehicle.</t>
+          <t>Julia and Miguel agreed the ladder should be quoted per vehicle ladder, with the bench sheet per vehicle.</t>
         </is>
       </c>
     </row>

</xml_diff>